<commit_message>
feat: add player skill card config and runtime skeleton
</commit_message>
<xml_diff>
--- a/Design/Excel/ET/Datas/Game/Hero.xlsx
+++ b/Design/Excel/ET/Datas/Game/Hero.xlsx
@@ -1,130 +1,48 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\ugit\myGameDevelopmentKit\Design\Excel\ET\Datas\Game\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10E08EBB-531F-4291-B078-3E29B5292D7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2280" yWindow="2280" windowWidth="19200" windowHeight="9970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2280" yWindow="2280" windowWidth="19200" windowHeight="9970" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
-  <si>
-    <t>##var</t>
-  </si>
-  <si>
-    <t>Id</t>
-  </si>
-  <si>
-    <t>##</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>ActiveSkill</t>
-  </si>
-  <si>
-    <t>PassiveSkill</t>
-  </si>
-  <si>
-    <t>##type</t>
-  </si>
-  <si>
-    <t>int</t>
-  </si>
-  <si>
-    <t>string</t>
-  </si>
-  <si>
-    <t>(array#sep=,),int</t>
-  </si>
-  <si>
-    <t>##group</t>
-  </si>
-  <si>
-    <t>c</t>
-  </si>
-  <si>
-    <t>策划备注</t>
-  </si>
-  <si>
-    <t>主动技能</t>
-  </si>
-  <si>
-    <t>被动技能</t>
-  </si>
-  <si>
-    <t>战士</t>
-  </si>
-  <si>
-    <t>1001,1002,1003,1004,1005,1006,1007,1008,1009,1010</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>int#ref=DTUnitConfig</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>UnitConfigId</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="等线"/>
       <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="3"/>
       <sz val="9"/>
-      <name val="等线"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -140,39 +58,99 @@
     </border>
   </borders>
   <cellStyleXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="常规 2" xfId="1" xr:uid="{8E7672AC-DA27-49A1-8A61-45C5BE1915EA}"/>
+    <cellStyle name="常规 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -433,104 +411,179 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="3" max="3" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.75" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.25" customWidth="1"/>
-    <col min="6" max="6" width="49.25" customWidth="1"/>
-    <col min="7" max="7" width="23" customWidth="1"/>
-    <col min="8" max="8" width="16.9140625" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" customWidth="1"/>
-    <col min="10" max="10" width="22.58203125" customWidth="1"/>
+    <col width="8.5" bestFit="1" customWidth="1" style="4" min="3" max="3"/>
+    <col width="18.75" bestFit="1" customWidth="1" style="4" min="4" max="4"/>
+    <col width="16.25" customWidth="1" style="4" min="5" max="5"/>
+    <col width="49.25" customWidth="1" style="4" min="6" max="6"/>
+    <col width="23" customWidth="1" style="4" min="7" max="7"/>
+    <col width="16.9140625" customWidth="1" style="4" min="8" max="8"/>
+    <col width="14.33203125" customWidth="1" style="4" min="9" max="9"/>
+    <col width="22.58203125" customWidth="1" style="4" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" t="s">
-        <v>5</v>
+    <row r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>##var</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="C1" s="0" t="inlineStr">
+        <is>
+          <t>##</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>UnitConfigId</t>
+        </is>
+      </c>
+      <c r="E1" s="0" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="F1" s="0" t="inlineStr">
+        <is>
+          <t>ActiveSkill</t>
+        </is>
+      </c>
+      <c r="G1" s="0" t="inlineStr">
+        <is>
+          <t>PassiveSkill</t>
+        </is>
+      </c>
+      <c r="H1" s="0" t="inlineStr">
+        <is>
+          <t>BattleCardConfigId</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>9</v>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>##type</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>int#ref=DTUnitConfig</t>
+        </is>
+      </c>
+      <c r="E2" s="0" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>(array#sep=,),int</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>(array#sep=,),int</t>
+        </is>
+      </c>
+      <c r="H2" s="0" t="inlineStr">
+        <is>
+          <t>int#ref=DTBattleCardConfig</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" t="s">
-        <v>11</v>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>##group</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="H3" s="0" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" t="s">
-        <v>14</v>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>##</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>DesignerNote</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t>ActiveSkillIds</t>
+        </is>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
+        <is>
+          <t>PassiveSkillIds</t>
+        </is>
+      </c>
+      <c r="H4" s="0" t="inlineStr">
+        <is>
+          <t>BattleCardConfigId</t>
+        </is>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B5">
+    <row r="5">
+      <c r="B5" s="0" t="n">
         <v>1001</v>
       </c>
-      <c r="C5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5">
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>战士</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="n">
         <v>1001</v>
       </c>
-      <c r="E5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>16</v>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>战士</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>1001,1002,1003,1004,1005,1006,1007,1008,1009,1010</t>
+        </is>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="H5" s="0" t="n">
+        <v>1001</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: reduce player deck to single sweep card
</commit_message>
<xml_diff>
--- a/Design/Excel/ET/Datas/Game/Hero.xlsx
+++ b/Design/Excel/ET/Datas/Game/Hero.xlsx
@@ -571,14 +571,10 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>1001,1002,1003,1004,1005,1006,1007,1008,1009,1010</t>
-        </is>
-      </c>
-      <c r="G5" s="0" t="inlineStr">
-        <is>
-          <t>2001</t>
-        </is>
-      </c>
+          <t>1001</t>
+        </is>
+      </c>
+      <c r="G5" s="0" t="inlineStr"/>
       <c r="H5" s="0" t="n">
         <v>1001</v>
       </c>

</xml_diff>

<commit_message>
fix: trigger 7001 damage on projectile reach
</commit_message>
<xml_diff>
--- a/Design/Excel/ET/Datas/Game/Hero.xlsx
+++ b/Design/Excel/ET/Datas/Game/Hero.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\ugit\myGameDevelopmentKit\Design\Excel\ET\Datas\Game\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75F735B0-5F2F-42CB-8B77-5A61174D7EA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BC69CC4-7C11-4F60-B57E-BBC3F9137FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4870" yWindow="790" windowWidth="19200" windowHeight="9970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5210" yWindow="1130" windowWidth="19200" windowHeight="9970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -82,7 +82,7 @@
     <t>战士</t>
   </si>
   <si>
-    <t>1001,7001</t>
+    <t>7001</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>

</xml_diff>

<commit_message>
feat: initialize player skills from hero config
</commit_message>
<xml_diff>
--- a/Design/Excel/ET/Datas/Game/Hero.xlsx
+++ b/Design/Excel/ET/Datas/Game/Hero.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\ugit\myGameDevelopmentKit\Design\Excel\ET\Datas\Game\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0155AB7D-4878-4E58-9E64-27EBB498F9B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA019BEF-1CEF-4381-BF35-78498A6BF7E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6490" yWindow="2940" windowWidth="19200" windowHeight="9970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2210" yWindow="2070" windowWidth="19200" windowHeight="9970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="24">
   <si>
     <t>##var</t>
   </si>
@@ -37,12 +37,6 @@
     <t>Name</t>
   </si>
   <si>
-    <t>ActiveSkill</t>
-  </si>
-  <si>
-    <t>PassiveSkill</t>
-  </si>
-  <si>
     <t>BattleCardConfigId</t>
   </si>
   <si>
@@ -73,9 +67,6 @@
     <t>ActiveSkillIds</t>
   </si>
   <si>
-    <t>PassiveSkillIds</t>
-  </si>
-  <si>
     <t>战士</t>
   </si>
   <si>
@@ -104,6 +95,10 @@
   </si>
   <si>
     <t>0_0_1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Skill</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -448,20 +443,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="8.5" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.75" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="16.25" style="4" customWidth="1"/>
-    <col min="7" max="7" width="49.25" style="4" customWidth="1"/>
-    <col min="8" max="8" width="23" style="4" customWidth="1"/>
-    <col min="9" max="9" width="24.08203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.33203125" style="4" customWidth="1"/>
-    <col min="11" max="11" width="22.58203125" style="4" customWidth="1"/>
+    <col min="7" max="7" width="23.75" style="4" customWidth="1"/>
+    <col min="8" max="8" width="24.08203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" style="4" customWidth="1"/>
+    <col min="10" max="10" width="22.58203125" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -478,97 +472,87 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="B2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>7</v>
       </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="G2" s="1" t="s">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="G3" t="s">
         <v>12</v>
       </c>
+      <c r="H3" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B5">
         <v>10001</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D5">
         <v>1001</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5"/>
-      <c r="I5">
+        <v>16</v>
+      </c>
+      <c r="H5">
         <v>1001</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B6">
         <v>10002</v>
       </c>
@@ -576,15 +560,15 @@
         <v>1001</v>
       </c>
       <c r="E6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I6" s="4">
+        <v>16</v>
+      </c>
+      <c r="H6" s="4">
         <v>1001</v>
       </c>
     </row>

</xml_diff>